<commit_message>
Tidy up, fixes and finishes
</commit_message>
<xml_diff>
--- a/active format script.xlsx
+++ b/active format script.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28227"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28429"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\benka\Desktop\לימודים\סמסטר ה\עיצוב צליל למשחקי מחשב\Final Project\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\nemne\Desktop\space\SoundDesign-for-VG-Course-Assignment\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{603E0F57-3F13-40F4-B7DA-C848BC9344C6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E7C4D92A-AAB6-44C2-A1E5-6AA0DAC57189}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="390" yWindow="390" windowWidth="21600" windowHeight="11295" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="v1" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="80" uniqueCount="64">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="88" uniqueCount="65">
   <si>
     <t>Character</t>
   </si>
@@ -85,9 +85,6 @@
     <t>Game Over screen</t>
   </si>
   <si>
-    <t>MIDI with editted with ReaSynth, added fade and Pan stereo effects</t>
-  </si>
-  <si>
     <t>gameOver.wav</t>
   </si>
   <si>
@@ -100,9 +97,6 @@
     <t>Menu screen</t>
   </si>
   <si>
-    <t>MIDI with Pan stereo effect</t>
-  </si>
-  <si>
     <t>menu.wav</t>
   </si>
   <si>
@@ -118,9 +112,6 @@
     <t>Level</t>
   </si>
   <si>
-    <t>ReaSynth with JS:Distortion effect and a tail to stay in rythm</t>
-  </si>
-  <si>
     <t>level.wav</t>
   </si>
   <si>
@@ -139,9 +130,6 @@
     <t xml:space="preserve">Foley with alternating crossfade </t>
   </si>
   <si>
-    <t>pauseMenu.wav</t>
-  </si>
-  <si>
     <t>Player</t>
   </si>
   <si>
@@ -175,9 +163,6 @@
     <t>Player taking damage</t>
   </si>
   <si>
-    <t>gotHit.wav</t>
-  </si>
-  <si>
     <t>Alien</t>
   </si>
   <si>
@@ -212,6 +197,24 @@
   </si>
   <si>
     <t>Foley with ReaXcomp, ReaGate, ReaNINJAM, ReaVerb</t>
+  </si>
+  <si>
+    <t>pause.wav</t>
+  </si>
+  <si>
+    <t>gotHit1.wav</t>
+  </si>
+  <si>
+    <t>gotHit2wav</t>
+  </si>
+  <si>
+    <t>MIDI with editted with ReaSynth, added fade and Pan stereo effects, Vital Synthesis, Stereo element</t>
+  </si>
+  <si>
+    <t>MIDI with Pan stereo effect, Vital Synthesis, Stereo element</t>
+  </si>
+  <si>
+    <t>ReaSynth with JS:Distortion effect and a tail to stay in rhythm, Magical8bit Synthesis, Stereo element</t>
   </si>
 </sst>
 </file>
@@ -274,10 +277,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
   </cellXfs>
@@ -617,19 +619,19 @@
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <dimension ref="A1:I10"/>
-  <sheetFormatPr defaultColWidth="12.6640625" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:H11"/>
+  <sheetFormatPr defaultColWidth="12.7109375" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="13.21875" customWidth="1"/>
-    <col min="2" max="2" width="25.88671875" customWidth="1"/>
-    <col min="3" max="3" width="43.21875" customWidth="1"/>
-    <col min="5" max="5" width="15.21875" customWidth="1"/>
-    <col min="6" max="6" width="17.6640625" customWidth="1"/>
-    <col min="7" max="7" width="58" customWidth="1"/>
-    <col min="8" max="8" width="14.33203125" customWidth="1"/>
+    <col min="1" max="1" width="13.28515625" customWidth="1"/>
+    <col min="2" max="2" width="25.85546875" customWidth="1"/>
+    <col min="3" max="3" width="43.28515625" customWidth="1"/>
+    <col min="5" max="5" width="15.28515625" customWidth="1"/>
+    <col min="6" max="6" width="17.7109375" customWidth="1"/>
+    <col min="7" max="7" width="94.42578125" customWidth="1"/>
+    <col min="8" max="8" width="14.28515625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -654,240 +656,265 @@
       <c r="H1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="2"/>
-    </row>
-    <row r="2" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="3" t="s">
+    </row>
+    <row r="2" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A2" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="B2" s="3" t="s">
+      <c r="B2" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="C2" s="3" t="s">
+      <c r="C2" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="E2" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="F2" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="G2" s="2" t="s">
+        <v>57</v>
+      </c>
+      <c r="H2" s="2" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A3" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="B3" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C3" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="D3" s="2" t="s">
+        <v>56</v>
+      </c>
+      <c r="E3" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="F3" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="G3" s="2" t="s">
+        <v>58</v>
+      </c>
+      <c r="H3" s="2" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A4" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="C4" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="D4" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="E4" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="F4" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="G4" s="2" t="s">
+        <v>62</v>
+      </c>
+      <c r="H4" s="2" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A5" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="B5" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="C5" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="D5" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="E5" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="F5" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="G5" s="2" t="s">
+        <v>63</v>
+      </c>
+      <c r="H5" s="2" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A6" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="B6" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="C6" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="D6" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="E6" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="F6" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="G6" s="2" t="s">
+        <v>64</v>
+      </c>
+      <c r="H6" s="2" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A7" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="B7" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="C7" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="D7" s="3" t="s">
+        <v>32</v>
+      </c>
+      <c r="E7" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="F7" s="3" t="s">
+        <v>34</v>
+      </c>
+      <c r="G7" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="H7" s="3" t="s">
         <v>59</v>
       </c>
-      <c r="D2" s="3" t="s">
+    </row>
+    <row r="8" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A8" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="B8" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="C8" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="D8" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="E8" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="F8" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="G8" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="H8" s="2" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A9" s="3" t="s">
+        <v>36</v>
+      </c>
+      <c r="B9" s="3" t="s">
         <v>43</v>
       </c>
-      <c r="E2" s="3" t="s">
-        <v>10</v>
-      </c>
-      <c r="F2" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="G2" s="3" t="s">
-        <v>62</v>
-      </c>
-      <c r="H2" s="3" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="3" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="B3" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="C3" s="3" t="s">
+      <c r="C9" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D9" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E9" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="F9" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="G9" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="H9" s="3" t="s">
         <v>60</v>
       </c>
-      <c r="D3" s="3" t="s">
+    </row>
+    <row r="10" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A10" s="3" t="s">
+        <v>36</v>
+      </c>
+      <c r="B10" s="3" t="s">
+        <v>43</v>
+      </c>
+      <c r="C10" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D10" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E10" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="F10" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="G10" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="H10" s="3" t="s">
         <v>61</v>
       </c>
-      <c r="E3" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="F3" s="3" t="s">
-        <v>15</v>
-      </c>
-      <c r="G3" s="3" t="s">
-        <v>63</v>
-      </c>
-      <c r="H3" s="3" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="4" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="B4" s="3" t="s">
-        <v>17</v>
-      </c>
-      <c r="C4" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="D4" s="3" t="s">
-        <v>19</v>
-      </c>
-      <c r="E4" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="F4" s="3" t="s">
-        <v>20</v>
-      </c>
-      <c r="G4" s="3" t="s">
-        <v>21</v>
-      </c>
-      <c r="H4" s="3" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="5" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="B5" s="3" t="s">
-        <v>17</v>
-      </c>
-      <c r="C5" s="3" t="s">
-        <v>23</v>
-      </c>
-      <c r="D5" s="3" t="s">
-        <v>24</v>
-      </c>
-      <c r="E5" s="3" t="s">
-        <v>10</v>
-      </c>
-      <c r="F5" s="3" t="s">
-        <v>25</v>
-      </c>
-      <c r="G5" s="3" t="s">
-        <v>26</v>
-      </c>
-      <c r="H5" s="3" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="6" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="B6" s="3" t="s">
-        <v>17</v>
-      </c>
-      <c r="C6" s="3" t="s">
+    </row>
+    <row r="11" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A11" s="2" t="s">
+        <v>47</v>
+      </c>
+      <c r="B11" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="C11" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="D11" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="E11" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="D6" s="3" t="s">
-        <v>29</v>
-      </c>
-      <c r="E6" s="3" t="s">
-        <v>30</v>
-      </c>
-      <c r="F6" s="3" t="s">
-        <v>31</v>
-      </c>
-      <c r="G6" s="3" t="s">
-        <v>32</v>
-      </c>
-      <c r="H6" s="3" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="7" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="4" t="s">
-        <v>8</v>
-      </c>
-      <c r="B7" s="4" t="s">
-        <v>17</v>
-      </c>
-      <c r="C7" s="4" t="s">
-        <v>34</v>
-      </c>
-      <c r="D7" s="4" t="s">
-        <v>35</v>
-      </c>
-      <c r="E7" s="4" t="s">
-        <v>36</v>
-      </c>
-      <c r="F7" s="4" t="s">
-        <v>37</v>
-      </c>
-      <c r="G7" s="4" t="s">
-        <v>38</v>
-      </c>
-      <c r="H7" s="4" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="8" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="3" t="s">
-        <v>40</v>
-      </c>
-      <c r="B8" s="3" t="s">
-        <v>41</v>
-      </c>
-      <c r="C8" s="3" t="s">
-        <v>42</v>
-      </c>
-      <c r="D8" s="3" t="s">
-        <v>43</v>
-      </c>
-      <c r="E8" s="3" t="s">
-        <v>30</v>
-      </c>
-      <c r="F8" s="3" t="s">
-        <v>44</v>
-      </c>
-      <c r="G8" s="3" t="s">
-        <v>45</v>
-      </c>
-      <c r="H8" s="3" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="9" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="4" t="s">
-        <v>40</v>
-      </c>
-      <c r="B9" s="4" t="s">
-        <v>47</v>
-      </c>
-      <c r="C9" s="4" t="s">
-        <v>48</v>
-      </c>
-      <c r="D9" s="4" t="s">
-        <v>49</v>
-      </c>
-      <c r="E9" s="4" t="s">
-        <v>30</v>
-      </c>
-      <c r="F9" s="4" t="s">
-        <v>50</v>
-      </c>
-      <c r="G9" s="4" t="s">
-        <v>12</v>
-      </c>
-      <c r="H9" s="4" t="s">
+      <c r="F11" s="2" t="s">
         <v>51</v>
       </c>
-    </row>
-    <row r="10" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="3" t="s">
+      <c r="G11" s="2" t="s">
         <v>52</v>
       </c>
-      <c r="B10" s="3" t="s">
+      <c r="H11" s="2" t="s">
         <v>53</v>
-      </c>
-      <c r="C10" s="3" t="s">
-        <v>54</v>
-      </c>
-      <c r="D10" s="3" t="s">
-        <v>55</v>
-      </c>
-      <c r="E10" s="3" t="s">
-        <v>30</v>
-      </c>
-      <c r="F10" s="3" t="s">
-        <v>56</v>
-      </c>
-      <c r="G10" s="3" t="s">
-        <v>57</v>
-      </c>
-      <c r="H10" s="3" t="s">
-        <v>58</v>
       </c>
     </row>
   </sheetData>

</xml_diff>